<commit_message>
changes: adding content has and timestamps
</commit_message>
<xml_diff>
--- a/Scraping scripts/nfk/nfk_nl_table.xlsx
+++ b/Scraping scripts/nfk/nfk_nl_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="131">
   <si>
     <t>Cancer_type</t>
   </si>
@@ -49,6 +49,9 @@
     <t>Date</t>
   </si>
   <si>
+    <t>Content_hash</t>
+  </si>
+  <si>
     <t>All / General</t>
   </si>
   <si>
@@ -184,7 +187,7 @@
     <t>NFK komt op voor een goede kwaliteit van het dagelijks leven voor mensen die leven met of na kanker en hun naasten, met ondersteuning om deel te nemen aan de samenleving.</t>
   </si>
   <si>
-    <t>Praktische hulpmiddelen en advies om een gezonde leefstijl te behouden tijdens en na de kankerbehandeling.</t>
+    <t>Praktische hulpmiddelen van en advies om een gezonde leefstijl te behouden tijdens en na de kankerbehandeling.</t>
   </si>
   <si>
     <t>NFK is de koepelorganisatie voor 22 kankerpatiëntenorganisaties die gerichte lotgenotenondersteuning en informatie bieden.</t>
@@ -364,7 +367,46 @@
     <t>contact, helpline, support</t>
   </si>
   <si>
-    <t>2026-05-25</t>
+    <t>2026-05-31 14:53:16</t>
+  </si>
+  <si>
+    <t>9c0f75b9a7742575bdd20b7c527feb2cf9e4388f2cd554ba96609e1bdb8316cb</t>
+  </si>
+  <si>
+    <t>f696c186fbb8df70dc58a95ae9bd7ccd154bf60a48c1c18fdf9fd09be3612cf2</t>
+  </si>
+  <si>
+    <t>c48541473ef898e3a07cf3aeab68abbdd8ebccd48fbcd5750293fad1e3b8be3c</t>
+  </si>
+  <si>
+    <t>9286008667d604ebb43d8bf1d0d3d5d97c9897a2f8d0300834fc144fc4be4c55</t>
+  </si>
+  <si>
+    <t>f6b51ba3531eddf56fc5b9c3fd225315e18e43904d829fb418440b79231c9a76</t>
+  </si>
+  <si>
+    <t>77dad81d5fa1a2527a816493effbed7bdcb5a7ab153696d796428931eb510340</t>
+  </si>
+  <si>
+    <t>6001c0688c9a35734e5506cc5858ff9350ed5f4fc9f115964aececdb90483add</t>
+  </si>
+  <si>
+    <t>dfed5411fef032e2863e42dbf5721c2f43343021b377eae95065f2f701b91c02</t>
+  </si>
+  <si>
+    <t>706713d462cb49ea3de4e7de66860d67237b3042989846facd696e28154fae5f</t>
+  </si>
+  <si>
+    <t>96a5c6a21668697e96b6944d9bf9a165607bb890e7974ca6a430d2c72dd3a17b</t>
+  </si>
+  <si>
+    <t>d7ac763f15097748747caadd1d16a6b3681f85dd368329c27bdda450f7bd3989</t>
+  </si>
+  <si>
+    <t>9895fa868dc691025c954f856403f0bcb3963c83eb399b7d2aa1a35ff700baaf</t>
+  </si>
+  <si>
+    <t>f553250c8cf0df267481fe325d39f89eb91d4d868fe1a207a91f3420793e992c</t>
   </si>
 </sst>
 </file>
@@ -735,10 +777,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -772,460 +814,502 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I2" t="s">
+        <v>91</v>
+      </c>
+      <c r="J2" t="s">
+        <v>104</v>
+      </c>
+      <c r="K2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I3" t="s">
+        <v>92</v>
+      </c>
+      <c r="J3" t="s">
+        <v>105</v>
+      </c>
+      <c r="K3" t="s">
+        <v>117</v>
+      </c>
+      <c r="L3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H4" t="s">
+        <v>86</v>
+      </c>
+      <c r="I4" t="s">
+        <v>93</v>
+      </c>
+      <c r="J4" t="s">
+        <v>106</v>
+      </c>
+      <c r="K4" t="s">
+        <v>117</v>
+      </c>
+      <c r="L4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G5" t="s">
+        <v>75</v>
+      </c>
+      <c r="H5" t="s">
+        <v>87</v>
+      </c>
+      <c r="I5" t="s">
+        <v>94</v>
+      </c>
+      <c r="J5" t="s">
+        <v>107</v>
+      </c>
+      <c r="K5" t="s">
+        <v>117</v>
+      </c>
+      <c r="L5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H6" t="s">
+        <v>84</v>
+      </c>
+      <c r="I6" t="s">
+        <v>95</v>
+      </c>
+      <c r="J6" t="s">
+        <v>108</v>
+      </c>
+      <c r="K6" t="s">
+        <v>117</v>
+      </c>
+      <c r="L6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" t="s">
+        <v>57</v>
+      </c>
+      <c r="F7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G7" t="s">
+        <v>77</v>
+      </c>
+      <c r="H7" t="s">
+        <v>88</v>
+      </c>
+      <c r="I7" t="s">
+        <v>96</v>
+      </c>
+      <c r="J7" t="s">
+        <v>109</v>
+      </c>
+      <c r="K7" t="s">
+        <v>117</v>
+      </c>
+      <c r="L7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E8" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" t="s">
+        <v>67</v>
+      </c>
+      <c r="G8" t="s">
+        <v>78</v>
+      </c>
+      <c r="H8" t="s">
+        <v>84</v>
+      </c>
+      <c r="I8" t="s">
+        <v>97</v>
+      </c>
+      <c r="J8" t="s">
+        <v>110</v>
+      </c>
+      <c r="K8" t="s">
+        <v>117</v>
+      </c>
+      <c r="L8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H9" t="s">
+        <v>89</v>
+      </c>
+      <c r="I9" t="s">
+        <v>98</v>
+      </c>
+      <c r="J9" t="s">
+        <v>111</v>
+      </c>
+      <c r="K9" t="s">
+        <v>117</v>
+      </c>
+      <c r="L9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" t="s">
+        <v>79</v>
+      </c>
+      <c r="H10" t="s">
+        <v>84</v>
+      </c>
+      <c r="I10" t="s">
+        <v>99</v>
+      </c>
+      <c r="J10" t="s">
+        <v>112</v>
+      </c>
+      <c r="K10" t="s">
+        <v>117</v>
+      </c>
+      <c r="L10" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F11" t="s">
+        <v>70</v>
+      </c>
+      <c r="G11" t="s">
+        <v>80</v>
+      </c>
+      <c r="H11" t="s">
+        <v>90</v>
+      </c>
+      <c r="I11" t="s">
+        <v>100</v>
+      </c>
+      <c r="J11" t="s">
+        <v>113</v>
+      </c>
+      <c r="K11" t="s">
+        <v>117</v>
+      </c>
+      <c r="L11" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" t="s">
+        <v>81</v>
+      </c>
+      <c r="H12" t="s">
+        <v>84</v>
+      </c>
+      <c r="I12" t="s">
+        <v>101</v>
+      </c>
+      <c r="J12" t="s">
+        <v>114</v>
+      </c>
+      <c r="K12" t="s">
+        <v>117</v>
+      </c>
+      <c r="L12" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G13" t="s">
+        <v>82</v>
+      </c>
+      <c r="H13" t="s">
+        <v>88</v>
+      </c>
+      <c r="I13" t="s">
+        <v>102</v>
+      </c>
+      <c r="J13" t="s">
+        <v>115</v>
+      </c>
+      <c r="K13" t="s">
+        <v>117</v>
+      </c>
+      <c r="L13" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D2" t="s">
+      <c r="C14" t="s">
         <v>38</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D14" t="s">
         <v>51</v>
       </c>
-      <c r="F2" t="s">
+      <c r="E14" t="s">
         <v>64</v>
       </c>
-      <c r="G2" t="s">
+      <c r="F14" t="s">
         <v>71</v>
       </c>
-      <c r="H2" t="s">
+      <c r="G14" t="s">
         <v>83</v>
       </c>
-      <c r="I2" t="s">
-        <v>90</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="H14" t="s">
+        <v>84</v>
+      </c>
+      <c r="I14" t="s">
         <v>103</v>
       </c>
-      <c r="K2" t="s">
+      <c r="J14" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G3" t="s">
-        <v>72</v>
-      </c>
-      <c r="H3" t="s">
-        <v>84</v>
-      </c>
-      <c r="I3" t="s">
-        <v>91</v>
-      </c>
-      <c r="J3" t="s">
-        <v>104</v>
-      </c>
-      <c r="K3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E4" t="s">
-        <v>53</v>
-      </c>
-      <c r="F4" t="s">
-        <v>66</v>
-      </c>
-      <c r="G4" t="s">
-        <v>73</v>
-      </c>
-      <c r="H4" t="s">
-        <v>85</v>
-      </c>
-      <c r="I4" t="s">
-        <v>92</v>
-      </c>
-      <c r="J4" t="s">
-        <v>105</v>
-      </c>
-      <c r="K4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E5" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" t="s">
-        <v>65</v>
-      </c>
-      <c r="G5" t="s">
-        <v>74</v>
-      </c>
-      <c r="H5" t="s">
-        <v>86</v>
-      </c>
-      <c r="I5" t="s">
-        <v>93</v>
-      </c>
-      <c r="J5" t="s">
-        <v>106</v>
-      </c>
-      <c r="K5" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F6" t="s">
-        <v>67</v>
-      </c>
-      <c r="G6" t="s">
-        <v>75</v>
-      </c>
-      <c r="H6" t="s">
-        <v>83</v>
-      </c>
-      <c r="I6" t="s">
-        <v>94</v>
-      </c>
-      <c r="J6" t="s">
-        <v>107</v>
-      </c>
-      <c r="K6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E7" t="s">
-        <v>56</v>
-      </c>
-      <c r="F7" t="s">
-        <v>68</v>
-      </c>
-      <c r="G7" t="s">
-        <v>76</v>
-      </c>
-      <c r="H7" t="s">
-        <v>87</v>
-      </c>
-      <c r="I7" t="s">
-        <v>95</v>
-      </c>
-      <c r="J7" t="s">
-        <v>108</v>
-      </c>
-      <c r="K7" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" t="s">
-        <v>57</v>
-      </c>
-      <c r="F8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G8" t="s">
-        <v>77</v>
-      </c>
-      <c r="H8" t="s">
-        <v>83</v>
-      </c>
-      <c r="I8" t="s">
-        <v>96</v>
-      </c>
-      <c r="J8" t="s">
-        <v>109</v>
-      </c>
-      <c r="K8" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" t="s">
-        <v>58</v>
-      </c>
-      <c r="F9" t="s">
-        <v>66</v>
-      </c>
-      <c r="G9" t="s">
-        <v>32</v>
-      </c>
-      <c r="H9" t="s">
-        <v>88</v>
-      </c>
-      <c r="I9" t="s">
-        <v>97</v>
-      </c>
-      <c r="J9" t="s">
-        <v>110</v>
-      </c>
-      <c r="K9" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" t="s">
-        <v>46</v>
-      </c>
-      <c r="E10" t="s">
-        <v>59</v>
-      </c>
-      <c r="F10" t="s">
-        <v>66</v>
-      </c>
-      <c r="G10" t="s">
-        <v>78</v>
-      </c>
-      <c r="H10" t="s">
-        <v>83</v>
-      </c>
-      <c r="I10" t="s">
-        <v>98</v>
-      </c>
-      <c r="J10" t="s">
-        <v>111</v>
-      </c>
-      <c r="K10" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11" t="s">
-        <v>69</v>
-      </c>
-      <c r="G11" t="s">
-        <v>79</v>
-      </c>
-      <c r="H11" t="s">
-        <v>89</v>
-      </c>
-      <c r="I11" t="s">
-        <v>99</v>
-      </c>
-      <c r="J11" t="s">
-        <v>112</v>
-      </c>
-      <c r="K11" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" t="s">
-        <v>48</v>
-      </c>
-      <c r="E12" t="s">
-        <v>61</v>
-      </c>
-      <c r="F12" t="s">
-        <v>66</v>
-      </c>
-      <c r="G12" t="s">
-        <v>80</v>
-      </c>
-      <c r="H12" t="s">
-        <v>83</v>
-      </c>
-      <c r="I12" t="s">
-        <v>100</v>
-      </c>
-      <c r="J12" t="s">
-        <v>113</v>
-      </c>
-      <c r="K12" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" t="s">
-        <v>49</v>
-      </c>
-      <c r="E13" t="s">
-        <v>62</v>
-      </c>
-      <c r="F13" t="s">
-        <v>68</v>
-      </c>
-      <c r="G13" t="s">
-        <v>81</v>
-      </c>
-      <c r="H13" t="s">
-        <v>87</v>
-      </c>
-      <c r="I13" t="s">
-        <v>101</v>
-      </c>
-      <c r="J13" t="s">
-        <v>114</v>
-      </c>
-      <c r="K13" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11">
-      <c r="A14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D14" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" t="s">
-        <v>63</v>
-      </c>
-      <c r="F14" t="s">
-        <v>70</v>
-      </c>
-      <c r="G14" t="s">
-        <v>82</v>
-      </c>
-      <c r="H14" t="s">
-        <v>83</v>
-      </c>
-      <c r="I14" t="s">
-        <v>102</v>
-      </c>
-      <c r="J14" t="s">
-        <v>115</v>
-      </c>
       <c r="K14" t="s">
-        <v>116</v>
+        <v>117</v>
+      </c>
+      <c r="L14" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>